<commit_message>
Dashboard update 2026-10-01 21:39
</commit_message>
<xml_diff>
--- a/excel/Afranga.xlsx
+++ b/excel/Afranga.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.08.08\Afranga\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19A36710-AEB7-416A-B209-B316617BD33E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E0F65D-053A-49A5-8F3E-C5B0D97458F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -406,7 +406,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -503,12 +503,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1974,43 +1968,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="43" t="s">
+      <c r="A1" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="46" t="s">
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="Q1" s="47" t="s">
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="Q1" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="48"/>
-      <c r="S1" s="48"/>
-      <c r="T1" s="49"/>
-      <c r="U1" s="47" t="s">
+      <c r="R1" s="46"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="47"/>
+      <c r="U1" s="45" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="49"/>
-      <c r="W1" s="43" t="s">
+      <c r="V1" s="47"/>
+      <c r="W1" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="X1" s="44"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="X1" s="42"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
       <c r="AA1" s="4" t="s">
         <v>39</v>
       </c>
@@ -2141,7 +2135,7 @@
       </c>
       <c r="K3" s="17">
         <f ca="1">'10000159'!B12</f>
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="L3" s="17" t="str">
         <f ca="1">'10000159'!P3</f>
@@ -2153,11 +2147,11 @@
       </c>
       <c r="N3" s="3">
         <f>'10000159'!L3</f>
-        <v>4.78</v>
+        <v>5.32</v>
       </c>
       <c r="O3" s="3">
         <f>'10000159'!M3</f>
-        <v>0.44999999999999996</v>
+        <v>0.49999999999999994</v>
       </c>
       <c r="P3" s="9"/>
       <c r="Q3" s="32">
@@ -2174,7 +2168,7 @@
       </c>
       <c r="T3" s="32">
         <f>W3-R3</f>
-        <v>0</v>
+        <v>2.3800000000000523</v>
       </c>
       <c r="U3" s="32">
         <f>SUM(M3:M100)</f>
@@ -2182,27 +2176,27 @@
       </c>
       <c r="V3" s="32">
         <f>SUM(N3:N100)-AA3</f>
-        <v>15.54</v>
+        <v>17.920000000000002</v>
       </c>
       <c r="W3" s="32">
         <f>Q3+V3+S3</f>
-        <v>317.41000000000003</v>
+        <v>319.79000000000002</v>
       </c>
       <c r="X3" s="32">
         <f>W3-Q3</f>
-        <v>17.410000000000025</v>
+        <v>19.79000000000002</v>
       </c>
       <c r="Y3" s="35">
         <f>(W3-Q3)/Q3</f>
-        <v>5.8033333333333416E-2</v>
+        <v>6.5966666666666729E-2</v>
       </c>
       <c r="Z3" s="35">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>9.4554528594017001E-2</v>
+        <v>9.4623056054115307E-2</v>
       </c>
       <c r="AA3" s="32">
         <f>SUM(O3:O100)</f>
-        <v>1.8</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="AC3" s="3" t="str">
         <f ca="1">'10000159'!Z3</f>
@@ -2251,7 +2245,7 @@
       </c>
       <c r="K4" s="17">
         <f ca="1">'10000160'!B12</f>
-        <v>245</v>
+        <v>215</v>
       </c>
       <c r="L4" s="17" t="str">
         <f ca="1">'10000160'!P3</f>
@@ -2263,11 +2257,11 @@
       </c>
       <c r="N4" s="3">
         <f>'10000160'!L3</f>
-        <v>0.63000000000000012</v>
+        <v>0.70000000000000018</v>
       </c>
       <c r="O4" s="3">
         <f>'10000160'!M3</f>
-        <v>0.09</v>
+        <v>9.9999999999999992E-2</v>
       </c>
       <c r="P4" s="9"/>
       <c r="Q4" s="36"/>
@@ -2394,7 +2388,7 @@
       </c>
       <c r="K6" s="17">
         <f ca="1">'10000170'!B12</f>
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="L6" s="17" t="str">
         <f ca="1">'10000170'!P3</f>
@@ -2406,11 +2400,11 @@
       </c>
       <c r="N6" s="3">
         <f>'10000170'!L3</f>
-        <v>4.12</v>
+        <v>4.59</v>
       </c>
       <c r="O6" s="3">
         <f>'10000170'!M3</f>
-        <v>0.44</v>
+        <v>0.49</v>
       </c>
       <c r="P6" s="9"/>
       <c r="AC6" s="3" t="str">
@@ -2460,7 +2454,7 @@
       </c>
       <c r="K7" s="17">
         <f ca="1">'10000212'!B12</f>
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="L7" s="17" t="str">
         <f ca="1">'10000212'!P3</f>
@@ -2472,11 +2466,11 @@
       </c>
       <c r="N7" s="3">
         <f>'10000212'!L3</f>
-        <v>1.5599999999999998</v>
+        <v>1.7599999999999998</v>
       </c>
       <c r="O7" s="3">
         <f>'10000212'!M3</f>
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="P7" s="9"/>
       <c r="AC7" s="3" t="str">
@@ -2526,7 +2520,7 @@
       </c>
       <c r="K8" s="17">
         <f ca="1">'10000263'!B12</f>
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="L8" s="17" t="str">
         <f ca="1">'10000263'!P3</f>
@@ -2538,11 +2532,11 @@
       </c>
       <c r="N8" s="3">
         <f>'10000263'!L3</f>
-        <v>1.18</v>
+        <v>1.3599999999999999</v>
       </c>
       <c r="O8" s="3">
         <f>'10000263'!M3</f>
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="P8" s="9"/>
       <c r="AC8" s="3" t="str">
@@ -2592,7 +2586,7 @@
       </c>
       <c r="K9" s="17">
         <f ca="1">'10000288'!B12</f>
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="L9" s="17" t="str">
         <f ca="1">'10000288'!P3</f>
@@ -2604,11 +2598,11 @@
       </c>
       <c r="N9" s="3">
         <f>'10000288'!L3</f>
-        <v>1.32</v>
+        <v>1.54</v>
       </c>
       <c r="O9" s="3">
         <f>'10000288'!M3</f>
-        <v>0.12000000000000001</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="P9" s="9"/>
       <c r="AC9" s="3" t="str">
@@ -2658,7 +2652,7 @@
       </c>
       <c r="K10" s="17">
         <f ca="1">'10000437'!B12</f>
-        <v>940</v>
+        <v>910</v>
       </c>
       <c r="L10" s="17" t="str">
         <f ca="1">'10000437'!P3</f>
@@ -2670,11 +2664,11 @@
       </c>
       <c r="N10" s="3">
         <f>'10000437'!L3</f>
-        <v>1.53</v>
+        <v>1.83</v>
       </c>
       <c r="O10" s="3">
         <f>'10000437'!M3</f>
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="P10" s="9"/>
       <c r="AC10" s="3" t="str">
@@ -2724,7 +2718,7 @@
       </c>
       <c r="K11" s="17">
         <f ca="1">'10000591'!B12</f>
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="L11" s="17" t="str">
         <f ca="1">'10000591'!P3</f>
@@ -2736,11 +2730,11 @@
       </c>
       <c r="N11" s="3">
         <f>'10000591'!L3</f>
-        <v>0.88</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="O11" s="3">
         <f>'10000591'!M3</f>
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="P11" s="9"/>
       <c r="AC11" s="3" t="str">
@@ -2856,7 +2850,7 @@
       </c>
       <c r="K13" s="17">
         <f ca="1">'10001244'!B12</f>
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="L13" s="17" t="str">
         <f ca="1">'10001244'!P3</f>
@@ -2868,11 +2862,11 @@
       </c>
       <c r="N13" s="3">
         <f>'10001244'!L3</f>
-        <v>0.23</v>
+        <v>0.43000000000000005</v>
       </c>
       <c r="O13" s="3">
         <f>'10001244'!M3</f>
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="AC13" s="3" t="str">
         <f ca="1">'10001244'!Z3</f>
@@ -2921,7 +2915,7 @@
       </c>
       <c r="K14" s="17">
         <f ca="1">'10001352'!B12</f>
-        <v>76</v>
+        <v>46</v>
       </c>
       <c r="L14" s="17" t="str">
         <f ca="1">'10001352'!P3</f>
@@ -2933,11 +2927,11 @@
       </c>
       <c r="N14" s="3">
         <f>'10001352'!L3</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="O14" s="3">
         <f>'10001352'!M3</f>
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="AC14" s="3" t="str">
         <f ca="1">'10001352'!Z3</f>
@@ -2986,7 +2980,7 @@
       </c>
       <c r="K15" s="17">
         <f ca="1">'10001457'!B12</f>
-        <v>380</v>
+        <v>350</v>
       </c>
       <c r="L15" s="17" t="str">
         <f ca="1">'10001457'!P3</f>
@@ -3079,16 +3073,16 @@
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
       <c r="O19" s="3"/>
-      <c r="Q19" s="40"/>
-      <c r="R19" s="40"/>
-      <c r="S19" s="40"/>
-      <c r="T19" s="40"/>
-      <c r="U19" s="40"/>
-      <c r="V19" s="40"/>
-      <c r="W19" s="40"/>
-      <c r="X19" s="40"/>
-      <c r="Y19" s="40"/>
-      <c r="Z19" s="40"/>
+      <c r="Q19" s="38"/>
+      <c r="R19" s="38"/>
+      <c r="S19" s="38"/>
+      <c r="T19" s="38"/>
+      <c r="U19" s="38"/>
+      <c r="V19" s="38"/>
+      <c r="W19" s="38"/>
+      <c r="X19" s="38"/>
+      <c r="Y19" s="38"/>
+      <c r="Z19" s="38"/>
       <c r="AA19" s="8"/>
       <c r="AC19" s="1"/>
     </row>
@@ -3270,7 +3264,7 @@
     <mergeCell ref="U1:V1"/>
     <mergeCell ref="W1:Z1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A16:N27 A3:O15">
+  <conditionalFormatting sqref="A3:O15 A16:N27">
     <cfRule type="expression" dxfId="57" priority="19">
       <formula>$AC3="+"</formula>
     </cfRule>
@@ -3343,29 +3337,29 @@
       <c r="B1" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -3457,11 +3451,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>1.18</v>
+        <v>1.3599999999999999</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -3672,14 +3666,22 @@
       <c r="D9" s="10">
         <v>46280</v>
       </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
+      <c r="E9" s="6">
+        <v>46280</v>
+      </c>
+      <c r="F9" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0.18</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0.02</v>
+      </c>
       <c r="J9" s="14"/>
       <c r="X9" s="6">
         <f t="shared" si="1"/>
@@ -3711,11 +3713,11 @@
       <c r="J10" s="14"/>
       <c r="X10" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46280</v>
       </c>
       <c r="Y10" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
@@ -3752,7 +3754,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="D12" s="10">
         <v>46371</v>
@@ -4622,11 +4624,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>1.18</v>
+        <v>1.3599999999999999</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
     </row>
   </sheetData>
@@ -4637,20 +4639,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="27" priority="1">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="2">
+    <cfRule type="expression" dxfId="22" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="25" priority="7">
+    <cfRule type="expression" dxfId="21" priority="7">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="24" priority="8">
+    <cfRule type="expression" dxfId="20" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4687,29 +4689,29 @@
       <c r="B1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -4801,11 +4803,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>1.5599999999999998</v>
+        <v>1.7599999999999998</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -5088,14 +5090,22 @@
       <c r="D11" s="10">
         <v>46284</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="E11" s="6">
+        <v>46284</v>
+      </c>
+      <c r="F11" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="3">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0.02</v>
+      </c>
       <c r="J11" s="14"/>
       <c r="X11" s="6">
         <f t="shared" si="1"/>
@@ -5112,7 +5122,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="D12" s="10">
         <v>46314</v>
@@ -5128,11 +5138,11 @@
       <c r="J12" s="14"/>
       <c r="X12" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46284</v>
       </c>
       <c r="Y12" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.18000000000000002</v>
       </c>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
@@ -5982,11 +5992,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>1.5599999999999998</v>
+        <v>1.7599999999999998</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
     </row>
   </sheetData>
@@ -5997,20 +6007,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="23" priority="1">
+    <cfRule type="expression" dxfId="19" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="21" priority="7">
+    <cfRule type="expression" dxfId="17" priority="7">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="20" priority="8">
+    <cfRule type="expression" dxfId="16" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6047,29 +6057,29 @@
       <c r="B1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -6161,11 +6171,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>4.12</v>
+        <v>4.59</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.44</v>
+        <v>0.49</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -6480,19 +6490,27 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="D12" s="10">
         <v>46279</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="E12" s="6">
+        <v>46279</v>
+      </c>
+      <c r="F12" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0.47</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.05</v>
+      </c>
       <c r="J12" s="14"/>
       <c r="X12" s="6">
         <f t="shared" si="1"/>
@@ -6521,11 +6539,11 @@
       <c r="N13" s="13"/>
       <c r="X13" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46279</v>
       </c>
       <c r="Y13" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
@@ -7350,11 +7368,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>4.12</v>
+        <v>4.59</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.44</v>
+        <v>0.49</v>
       </c>
     </row>
   </sheetData>
@@ -7365,20 +7383,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="19" priority="1">
+    <cfRule type="expression" dxfId="15" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="17" priority="7">
+    <cfRule type="expression" dxfId="13" priority="7">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="16" priority="8">
+    <cfRule type="expression" dxfId="12" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7418,29 +7436,29 @@
       <c r="B1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -8730,20 +8748,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="15" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="13" priority="7">
+    <cfRule type="expression" dxfId="9" priority="7">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="12" priority="8">
+    <cfRule type="expression" dxfId="8" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8780,29 +8798,29 @@
       <c r="B1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -8894,11 +8912,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.63000000000000012</v>
+        <v>0.70000000000000018</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.09</v>
+        <v>9.9999999999999992E-2</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -9213,19 +9231,27 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>245</v>
+        <v>215</v>
       </c>
       <c r="D12" s="10">
         <v>46268</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="E12" s="6">
+        <v>46268</v>
+      </c>
+      <c r="F12" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.01</v>
+      </c>
       <c r="J12" s="14"/>
       <c r="X12" s="6">
         <f t="shared" si="1"/>
@@ -9254,11 +9280,11 @@
       <c r="N13" s="13"/>
       <c r="X13" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46268</v>
       </c>
       <c r="Y13" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>6.0000000000000005E-2</v>
       </c>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
@@ -10095,11 +10121,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.63000000000000012</v>
+        <v>0.70000000000000018</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.09</v>
+        <v>9.9999999999999992E-2</v>
       </c>
     </row>
   </sheetData>
@@ -10110,20 +10136,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="9" priority="7">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="8" priority="8">
+    <cfRule type="expression" dxfId="4" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10160,29 +10186,29 @@
       <c r="B1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -10274,11 +10300,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>4.78</v>
+        <v>5.32</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.44999999999999996</v>
+        <v>0.49999999999999994</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -10593,19 +10619,27 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="D12" s="10">
         <v>46268</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="E12" s="6">
+        <v>46268</v>
+      </c>
+      <c r="F12" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0.54</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.05</v>
+      </c>
       <c r="J12" s="14"/>
       <c r="X12" s="6">
         <f t="shared" si="1"/>
@@ -10634,11 +10668,11 @@
       <c r="N13" s="13"/>
       <c r="X13" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46268</v>
       </c>
       <c r="Y13" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.49000000000000005</v>
       </c>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
@@ -11463,11 +11497,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>4.78</v>
+        <v>5.32</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.44999999999999996</v>
+        <v>0.49999999999999994</v>
       </c>
     </row>
   </sheetData>
@@ -11479,20 +11513,20 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="5" priority="5">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="4" priority="8">
+    <cfRule type="expression" dxfId="0" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13090,14 +13124,14 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="6">
         <f ca="1">TODAY()</f>
-        <v>46265</v>
+        <v>46295</v>
       </c>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
       <c r="D200" s="1"/>
       <c r="K200" s="28">
         <f>Overview!W3</f>
-        <v>317.41000000000003</v>
+        <v>319.79000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -13132,29 +13166,29 @@
       <c r="B1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -13163,53 +13197,53 @@
       <c r="B2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="39" t="s">
+      <c r="E2" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="F2" s="38" t="s">
+      <c r="F2" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="G2" s="39" t="s">
+      <c r="G2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="39" t="s">
+      <c r="H2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="39" t="s">
+      <c r="I2" s="11" t="s">
         <v>43</v>
       </c>
       <c r="J2" s="9"/>
-      <c r="K2" s="39" t="s">
-        <v>0</v>
-      </c>
-      <c r="L2" s="39" t="s">
+      <c r="K2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="L2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="39" t="s">
+      <c r="M2" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="N2" s="39" t="s">
+      <c r="N2" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="39" t="s">
+      <c r="O2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="P2" s="39" t="s">
+      <c r="P2" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="Q2" s="39" t="s">
+      <c r="Q2" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="X2" s="39" t="s">
+      <c r="X2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="Y2" s="39" t="s">
+      <c r="Y2" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="Z2" s="39" t="s">
+      <c r="Z2" s="11" t="s">
         <v>49</v>
       </c>
     </row>
@@ -13474,7 +13508,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>380</v>
+        <v>350</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -14353,20 +14387,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="51" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="50" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="49" priority="3">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="48" priority="4">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14403,29 +14437,29 @@
       <c r="B1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -14494,14 +14528,22 @@
       <c r="D3" s="10">
         <v>46280</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="17" t="str">
+      <c r="E3" s="10">
+        <v>46280</v>
+      </c>
+      <c r="F3" s="17">
         <f>IF(E3&gt;0,E3-D3,"")</f>
-        <v/>
-      </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0.03</v>
+      </c>
       <c r="J3" s="14"/>
       <c r="K3" s="3">
         <f>G53</f>
@@ -14509,11 +14551,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -14563,11 +14605,11 @@
       <c r="J4" s="9"/>
       <c r="X4" s="6">
         <f>E3</f>
-        <v>0</v>
+        <v>46280</v>
       </c>
       <c r="Y4" s="3">
         <f>G3+H3-I3</f>
-        <v>0</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
@@ -14749,7 +14791,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>76</v>
+        <v>46</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -15613,11 +15655,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>
@@ -15628,20 +15670,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="51" priority="1">
+    <cfRule type="expression" dxfId="47" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="50" priority="2">
+    <cfRule type="expression" dxfId="46" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="49" priority="3">
+    <cfRule type="expression" dxfId="45" priority="3">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="48" priority="4">
+    <cfRule type="expression" dxfId="44" priority="4">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15678,29 +15720,29 @@
       <c r="B1" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -15792,11 +15834,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.23</v>
+        <v>0.43000000000000005</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -15838,11 +15880,21 @@
       <c r="D4" s="10">
         <v>46280</v>
       </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="E4" s="10">
+        <v>46280</v>
+      </c>
+      <c r="F4" s="17">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0.02</v>
+      </c>
       <c r="J4" s="9"/>
       <c r="X4" s="6">
         <f>E3</f>
@@ -15870,11 +15922,11 @@
       <c r="J5" s="9"/>
       <c r="X5" s="6">
         <f t="shared" ref="X5:X52" si="1">E4</f>
-        <v>0</v>
+        <v>46280</v>
       </c>
       <c r="Y5" s="3">
         <f t="shared" ref="Y5:Y52" si="2">G4+H4-I4</f>
-        <v>0</v>
+        <v>0.18000000000000002</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
@@ -16032,7 +16084,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -16896,11 +16948,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.23</v>
+        <v>0.43000000000000005</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
     </row>
   </sheetData>
@@ -16911,20 +16963,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="47" priority="1">
+    <cfRule type="expression" dxfId="43" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="46" priority="2">
+    <cfRule type="expression" dxfId="42" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="45" priority="3">
+    <cfRule type="expression" dxfId="41" priority="3">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="44" priority="4">
+    <cfRule type="expression" dxfId="40" priority="4">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16964,29 +17016,29 @@
       <c r="B1" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -18216,20 +18268,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="43" priority="1">
+    <cfRule type="expression" dxfId="39" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="2">
+    <cfRule type="expression" dxfId="38" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="41" priority="3">
+    <cfRule type="expression" dxfId="37" priority="3">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="40" priority="4">
+    <cfRule type="expression" dxfId="36" priority="4">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18266,29 +18318,29 @@
       <c r="B1" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -18380,11 +18432,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.88</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -18522,14 +18574,22 @@
       <c r="D7" s="10">
         <v>46293</v>
       </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="E7" s="10">
+        <v>46293</v>
+      </c>
+      <c r="F7" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.22</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0.02</v>
+      </c>
       <c r="J7" s="14"/>
       <c r="X7" s="6">
         <f t="shared" si="1"/>
@@ -18562,11 +18622,11 @@
       <c r="J8" s="9"/>
       <c r="X8" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46293</v>
       </c>
       <c r="Y8" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
@@ -18659,7 +18719,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="D12" s="10">
         <v>46446</v>
@@ -19529,11 +19589,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.88</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -19544,20 +19604,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="39" priority="1">
+    <cfRule type="expression" dxfId="35" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="2">
+    <cfRule type="expression" dxfId="34" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="37" priority="9">
+    <cfRule type="expression" dxfId="33" priority="9">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="36" priority="10">
+    <cfRule type="expression" dxfId="32" priority="10">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19594,29 +19654,29 @@
       <c r="B1" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -19708,11 +19768,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>1.53</v>
+        <v>1.83</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -19886,14 +19946,22 @@
       <c r="D8" s="10">
         <v>46293</v>
       </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="2"/>
+      <c r="E8" s="6">
+        <v>46293</v>
+      </c>
+      <c r="F8" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="3">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0.03</v>
+      </c>
       <c r="J8" s="9"/>
       <c r="X8" s="6">
         <f t="shared" si="1"/>
@@ -19925,11 +19993,11 @@
       <c r="J9" s="14"/>
       <c r="X9" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46293</v>
       </c>
       <c r="Y9" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
@@ -19994,7 +20062,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>940</v>
+        <v>910</v>
       </c>
       <c r="D12" s="10">
         <v>46415</v>
@@ -20912,11 +20980,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>1.53</v>
+        <v>1.83</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
     </row>
   </sheetData>
@@ -20927,20 +20995,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="35" priority="1">
+    <cfRule type="expression" dxfId="31" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="2">
+    <cfRule type="expression" dxfId="30" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="33" priority="7">
+    <cfRule type="expression" dxfId="29" priority="7">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="32" priority="8">
+    <cfRule type="expression" dxfId="28" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20977,29 +21045,29 @@
       <c r="B1" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="45"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43"/>
+      <c r="X1" s="41"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -21091,11 +21159,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>1.32</v>
+        <v>1.54</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.12000000000000001</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -21306,14 +21374,22 @@
       <c r="D9" s="10">
         <v>46280</v>
       </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
+      <c r="E9" s="6">
+        <v>46280</v>
+      </c>
+      <c r="F9" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0.22</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0.02</v>
+      </c>
       <c r="J9" s="14"/>
       <c r="X9" s="6">
         <f t="shared" si="1"/>
@@ -21345,11 +21421,11 @@
       <c r="J10" s="14"/>
       <c r="X10" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46280</v>
       </c>
       <c r="Y10" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
@@ -21386,7 +21462,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="D12" s="10">
         <v>46371</v>
@@ -22256,11 +22332,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>1.32</v>
+        <v>1.54</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.12000000000000001</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -22271,20 +22347,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="31" priority="1">
+    <cfRule type="expression" dxfId="27" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="2">
+    <cfRule type="expression" dxfId="26" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="29" priority="7">
+    <cfRule type="expression" dxfId="25" priority="7">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="28" priority="8">
+    <cfRule type="expression" dxfId="24" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>